<commit_message>
Update carousel-log: Topic 4 entries
</commit_message>
<xml_diff>
--- a/carousel-data/carousel-log.xlsx
+++ b/carousel-data/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K129"/>
+  <dimension ref="A1:K132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7186,7 +7186,6 @@
           <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr">
         <is>
           <t>Strategic Planning Facilitator | Author</t>
@@ -7237,7 +7236,6 @@
           <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr">
         <is>
           <t>Strategic Planning Facilitator | Author</t>
@@ -7288,7 +7286,6 @@
           <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr">
         <is>
           <t>Strategic Planning Facilitator | Author</t>
@@ -7307,6 +7304,159 @@
       <c r="K129" t="inlineStr">
         <is>
           <t>Pain Point - How to Break the Cycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>why-worklife</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>https://consultclarity.org/post/podcast-rec-worklife-adam-grant</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>8</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousel-output/worklife-adam-grant</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Strategic Planning Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Podcast Rec - Why Every Leader Should Listen to WorkLife</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>worklife-lessons</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>https://consultclarity.org/post/podcast-rec-worklife-adam-grant</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>8</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousel-output/worklife-adam-grant</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Strategic Planning Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Podcast Rec - 5 Leadership Lessons from WorkLife</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>start-here-worklife</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>https://consultclarity.org/post/podcast-rec-worklife-adam-grant</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>8</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousel-output/worklife-adam-grant</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Strategic Planning Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Podcast Rec - New to WorkLife? Start Here</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update carousel-log.xlsx - Topic 3 Working Genius
</commit_message>
<xml_diff>
--- a/carousel-data/carousel-log.xlsx
+++ b/carousel-data/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K132"/>
+  <dimension ref="A1:K135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7336,7 +7336,6 @@
           <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr">
         <is>
           <t>Strategic Planning Facilitator | Author</t>
@@ -7387,7 +7386,6 @@
           <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr">
         <is>
           <t>Strategic Planning Facilitator | Author</t>
@@ -7438,7 +7436,6 @@
           <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr">
         <is>
           <t>Strategic Planning Facilitator | Author</t>
@@ -7457,6 +7454,171 @@
       <c r="K132" t="inlineStr">
         <is>
           <t>Podcast Rec - New to WorkLife? Start Here</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Working Genius: 6 Types That Energise or Drain You</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>6-types-of-working-genius</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>8</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>square, portrait, vertical</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>working-genius-6-types-2026-03-27/6-types-of-working-genius</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Working Genius: 6 Types That Energise or Drain You</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>why-your-team-feels-stuck</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>8</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>square, portrait, vertical</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>working-genius-6-types-2026-03-27/why-your-team-feels-stuck</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Working Genius: 6 Types That Energise or Drain You</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>genius-competency-frustration</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>8</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>square, portrait, vertical</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>working-genius-6-types-2026-03-27/genius-competency-frustration</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update carousel-log.xlsx - Topic 4 Five Dysfunctions
</commit_message>
<xml_diff>
--- a/carousel-data/carousel-log.xlsx
+++ b/carousel-data/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K135"/>
+  <dimension ref="A1:K138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7622,6 +7622,171 @@
         </is>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>The Five Dysfunctions of a Team (Summary)</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>five-dysfunctions-overview</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>8</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>square, portrait, vertical</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>five-dysfunctions-team-2026-03-27/five-dysfunctions-overview</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>The Five Dysfunctions of a Team (Summary)</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>signs-team-dysfunctional</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>8</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>square, portrait, vertical</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>five-dysfunctions-team-2026-03-27/signs-team-dysfunctional</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>The Five Dysfunctions of a Team (Summary)</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>building-cohesive-team</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>8</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>square, portrait, vertical</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>five-dysfunctions-team-2026-03-27/building-cohesive-team</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel log - 3 Crucial Conversations carousels
</commit_message>
<xml_diff>
--- a/carousel-data/carousel-log.xlsx
+++ b/carousel-data/carousel-log.xlsx
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -59,11 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K138"/>
+  <dimension ref="A1:K158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7160,7 +7163,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>priorities-just-words</t>
+          <t>why-priorities-fail</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -7170,7 +7173,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>https://consultclarity.org/post/every-year-we-set-priorities-and-do-the-same-things</t>
+          <t>N/A - Pain Point</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -7178,17 +7181,22 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>https://github.com/jonno-alt/social-images/tree/main/carousel-output/priorities-same-things</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/priorities-same-things-2026-03-26/why-priorities-fail</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+          <t>LI, FB, IG, Threads, X, GBP, TikTok, YT, Bluesky</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>Strategic Planning Facilitator | Author</t>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -7198,19 +7206,19 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Pain Point - 5 Signs Your Priorities Are Just Words</t>
+          <t>Pain point topic, no people to tag</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>why-teams-repeat</t>
+          <t>signs-plan-will-fail</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -7220,25 +7228,30 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>https://consultclarity.org/post/every-year-we-set-priorities-and-do-the-same-things</t>
+          <t>N/A - Pain Point</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>https://github.com/jonno-alt/social-images/tree/main/carousel-output/priorities-same-things</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/priorities-same-things-2026-03-26/signs-plan-will-fail</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+          <t>LI, FB, IG, Threads, X, GBP, TikTok, YT, Bluesky</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>Strategic Planning Facilitator | Author</t>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -7248,12 +7261,12 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>Pain Point - Why Teams Keep Doing the Same Things</t>
+          <t>Pain point topic, no people to tag</t>
         </is>
       </c>
     </row>
@@ -7270,7 +7283,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>https://consultclarity.org/post/every-year-we-set-priorities-and-do-the-same-things</t>
+          <t>N/A - Pain Point</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -7278,17 +7291,22 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>https://github.com/jonno-alt/social-images/tree/main/carousel-output/priorities-same-things</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/priorities-same-things-2026-03-26/break-the-cycle</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+          <t>IG, GBP, TikTok, YT (LI/FB/Threads/X/Bluesky failed)</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>LI, FB, Threads, X, Bluesky</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>Strategic Planning Facilitator | Author</t>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -7298,19 +7316,19 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>Pain Point - How to Break the Cycle</t>
+          <t>Pain point topic, no people to tag</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>why-worklife</t>
+          <t>worklife-podcast-rec</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -7320,7 +7338,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>https://consultclarity.org/post/podcast-rec-worklife-adam-grant</t>
+          <t>https://www.yourthoughtpartner.com/blog/worklife-with-adam-grant-podcast</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -7328,17 +7346,17 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>https://github.com/jonno-alt/social-images/tree/main/carousel-output/worklife-adam-grant</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/worklife-adam-grant-2026-03-26/worklife-podcast-rec</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>Strategic Planning Facilitator | Author</t>
+          <t>Founder, Clarity Group Global</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -7353,14 +7371,14 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Podcast Rec - Why Every Leader Should Listen to WorkLife</t>
+          <t>All 9 platforms scheduled. @adamgrant tagged on Instagram.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>worklife-lessons</t>
+          <t>worklife-why-listen</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -7370,25 +7388,25 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>https://consultclarity.org/post/podcast-rec-worklife-adam-grant</t>
+          <t>https://www.yourthoughtpartner.com/blog/worklife-with-adam-grant-podcast</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>https://github.com/jonno-alt/social-images/tree/main/carousel-output/worklife-adam-grant</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/worklife-adam-grant-2026-03-26/worklife-why-listen</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>Strategic Planning Facilitator | Author</t>
+          <t>Founder, Clarity Group Global</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -7403,24 +7421,19 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Podcast Rec - 5 Leadership Lessons from WorkLife</t>
+          <t>All 9 platforms scheduled. 5 Reasons Leaders Should Listen theme.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>start-here-worklife</t>
+          <t>keynote-speaking-service</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>https://consultclarity.org/post/podcast-rec-worklife-adam-grant</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7428,17 +7441,17 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>https://github.com/jonno-alt/social-images/tree/main/carousel-output/worklife-adam-grant</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/keynote-speaking-2026-03-26/keynote-speaking-service</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>Strategic Planning Facilitator | Author</t>
+          <t>Founder, Clarity Group Global</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -7453,337 +7466,1282 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Podcast Rec - New to WorkLife? Start Here</t>
+          <t>6 keynote topics overview. All 9 platforms.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
+          <t>why-book-jonno</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>Working Genius: 6 Types That Energise or Drain You</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="D133" t="inlineStr">
-        <is>
-          <t>6-types-of-working-genius</t>
-        </is>
-      </c>
-      <c r="E133" t="n">
-        <v>8</v>
+      <c r="D133" t="n">
+        <v>7</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/keynote-speaking-2026-03-26/why-book-jonno</t>
+        </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>square, portrait, vertical</t>
-        </is>
-      </c>
-      <c r="G133" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Founder, Clarity Group Global</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>working-genius-6-types-2026-03-27/6-types-of-working-genius</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>Certified Working Genius Facilitator | Author</t>
+          <t>5 reasons to book Jonno. All 9 platforms.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
+          <t>exec-team-dysfunction</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>Working Genius: 6 Types That Energise or Drain You</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr">
-        <is>
-          <t>why-your-team-feels-stuck</t>
-        </is>
-      </c>
-      <c r="E134" t="n">
-        <v>8</v>
+      <c r="D134" t="n">
+        <v>9</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/exec-team-dysfunction-2026-03-26/exec-team-dysfunction</t>
+        </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>square, portrait, vertical</t>
-        </is>
-      </c>
-      <c r="G134" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Founder, Clarity Group Global</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>working-genius-6-types-2026-03-27/why-your-team-feels-stuck</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>Certified Working Genius Facilitator | Author</t>
+          <t>7 signs of dysfunction. Lencioni framework. All 9 platforms.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
+          <t>fix-dysfunctional-team</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>Working Genius: 6 Types That Energise or Drain You</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="D135" t="inlineStr">
-        <is>
-          <t>genius-competency-frustration</t>
-        </is>
-      </c>
-      <c r="E135" t="n">
-        <v>8</v>
+      <c r="D135" t="n">
+        <v>7</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/exec-team-dysfunction-2026-03-26/fix-dysfunctional-team</t>
+        </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>square, portrait, vertical</t>
-        </is>
-      </c>
-      <c r="G135" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Founder, Clarity Group Global</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>working-genius-6-types-2026-03-27/genius-competency-frustration</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>Certified Working Genius Facilitator | Author</t>
+          <t>5 steps to high performance. Lencioni framework. All 9 platforms.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
+          <t>asba-93-percent-proof</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>The Five Dysfunctions of a Team (Summary)</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="D136" t="inlineStr">
-        <is>
-          <t>five-dysfunctions-overview</t>
-        </is>
-      </c>
-      <c r="E136" t="n">
+      <c r="D136" t="n">
         <v>8</v>
       </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/asba-93-percent-proof-2026-03-27</t>
+        </is>
+      </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>square, portrait, vertical</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>YouTube (disconnected), Google Business (disconnected)</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Certified Working Genius Facilitator | Author</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>five-dysfunctions-team-2026-03-27/five-dysfunctions-overview</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+          <t>Stats/proof topic about ASBA 2025 conference results</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
+          <t>asba-what-makes-pd-great</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>The Five Dysfunctions of a Team (Summary)</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="D137" t="inlineStr">
-        <is>
-          <t>signs-team-dysfunctional</t>
-        </is>
-      </c>
-      <c r="E137" t="n">
+      <c r="D137" t="n">
         <v>8</v>
       </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/asba-what-makes-pd-great-2026-03-27</t>
+        </is>
+      </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>square, portrait, vertical</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>YouTube (disconnected), Google Business (disconnected)</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Certified Working Genius Facilitator | Author</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>five-dysfunctions-team-2026-03-27/signs-team-dysfunctional</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+          <t>5 reasons Working Genius PD stands out</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
+          <t>extreme-ownership-why-read</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>The Five Dysfunctions of a Team (Summary)</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>building-cohesive-team</t>
-        </is>
-      </c>
-      <c r="E138" t="n">
+      <c r="D138" t="n">
         <v>8</v>
       </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/extreme-ownership-why-read-2026-03-27</t>
+        </is>
+      </c>
       <c r="F138" t="inlineStr">
         <is>
+          <t>LI,FB,IG,Threads,X,Bluesky,TikTok</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>YouTube,GBP (disconnected)</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Why read Extreme Ownership</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>extreme-ownership-principles</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>8</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/extreme-ownership-principles-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>LI,FB,IG,Threads,X,Bluesky,TikTok</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>YouTube,GBP (disconnected)</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>5 key principles</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>extreme-ownership-apply</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>7</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/extreme-ownership-apply-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>LI,FB,IG,Threads,X,Bluesky,TikTok</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>YouTube,GBP (disconnected)</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>How to apply</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>perfect-meeting-danger</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>8</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/perfect-meeting-danger-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>YouTube, Google Business</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>Pain point topic, no people to tag</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>perfect-meeting-fix</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>8</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/perfect-meeting-fix-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>YouTube, Google Business</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>Pain point topic, no people to tag</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>learning-leader-rec</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>8</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/learning-leader-rec-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>YouTube, Google Business</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>Podcast recommendation overview, tags @ryanhawk12</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>learning-leader-lessons</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>8</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/learning-leader-lessons-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>YouTube, Google Business</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>5 leadership lessons from the show, tags @ryanhawk12</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>offsite-insights-edward-amey</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="D145" t="n">
+        <v>8</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/testimonial-edward-amey-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Testimonial topic. Content from EP225 podcast and public bio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>leadership-disability-edward-amey</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="D146" t="n">
+        <v>7</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/testimonial-edward-amey-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Testimonial topic. Content from EP225 podcast and public bio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>why-leaders-need-a-coach</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="D147" t="n">
+        <v>8</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/service-executive-coaching-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Leadership Coach | Author</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>Service promo: Executive Coaching for Leaders</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>what-coaching-looks-like</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="D148" t="n">
+        <v>8</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/service-executive-coaching-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Leadership Coach | Author</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Service promo: Executive Coaching for Leaders</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>cost-of-no-coach</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="D149" t="n">
+        <v>8</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/service-executive-coaching-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Leadership Coach | Author</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Service promo: Executive Coaching for Leaders</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>wg-6-types</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>N/A - Framework topic</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>8</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/working-genius-6-types-2026-03-27/wg-6-types</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Working Genius: 6 Types Explained</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>wg-genius-or-frustration</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>N/A - Framework topic</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>8</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/working-genius-6-types-2026-03-27/wg-genius-or-frustration</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Genius, Competency, or Frustration</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>wg-transforms-teams</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>N/A - Framework topic</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>8</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/working-genius-6-types-2026-03-27/wg-transforms-teams</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>How Working Genius Transforms Teams</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>5d-overview</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>N/A - Book summary</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>8</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/five-dysfunctions-team-2026-03-27/5d-overview</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>All 9 platforms</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Five Dysfunctions Overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>5d-overcome</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>N/A - Book summary</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>8</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/five-dysfunctions-team-2026-03-27/5d-overcome</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>All 9 platforms</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>How to Overcome</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>5d-warning-signs</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>N/A - Book summary</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>8</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/five-dysfunctions-team-2026-03-27/5d-warning-signs</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>All 9 platforms</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>Warning Signs</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>crucial-conversations-overview</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Crucial Conversations by Patterson et al</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>6</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
           <t>square, portrait, vertical</t>
         </is>
       </c>
-      <c r="G138" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H138" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I138" t="inlineStr">
-        <is>
-          <t>five-dysfunctions-team-2026-03-27/building-cohesive-team</t>
-        </is>
-      </c>
-      <c r="J138" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="K138" t="inlineStr">
-        <is>
-          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Book overview, 3 defining elements, pool of shared meaning, conditions for dialogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>crucial-conversations-state-method</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Crucial Conversations by Patterson et al</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>7</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>square, portrait, vertical</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>STATE method: Share facts, Tell story, Ask others paths, Talk tentatively, Encourage testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>crucial-conversations-crib-technique</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Crucial Conversations by Patterson et al</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>7</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>square, portrait, vertical</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>CRIB technique: Commit, Recognize, Invent, Brainstorm for finding mutual purpose</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update carousel log - 3 Best Teacher Resigned carousels
</commit_message>
<xml_diff>
--- a/carousel-data/carousel-log.xlsx
+++ b/carousel-data/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K158"/>
+  <dimension ref="A1:K161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8745,6 +8745,126 @@
         </is>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>best-teacher-resigned-warning-signs</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Your Best Teacher Just Resigned</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>6</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>square, portrait, vertical</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>5 warning signs you missed, 75% stat, stay conversation advice</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>best-teacher-resigned-why-they-leave</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Your Best Teacher Just Resigned</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>6</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>square, portrait, vertical</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Real reasons: invisible, bureaucracy, no voice, toxic culture, no future. $10-20K cost per teacher</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>best-teacher-resigned-how-to-keep</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Your Best Teacher Just Resigned</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>7</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>square, portrait, vertical</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>6 strategies: relationships, voice, growth, protect time. 2/3 nobody asked them to stay</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx — session 2026-03-27 (4 topics)
</commit_message>
<xml_diff>
--- a/carousel-data/carousel-log.xlsx
+++ b/carousel-data/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K161"/>
+  <dimension ref="A1:K174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8628,240 +8628,915 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>crucial-conversations-overview</t>
+          <t>crucial-conversations-why-read</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Crucial Conversations by Patterson et al</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>square, portrait, vertical</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/crucial-conversations-book-rec-2026-03-27/crucial-conversations-why-read</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G156" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>Book overview, 3 defining elements, pool of shared meaning, conditions for dialogue</t>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>Book rec carousel. No people tagged.</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>crucial-conversations-state-method</t>
+          <t>crucial-conversations-7-skills</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Crucial Conversations by Patterson et al</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>square, portrait, vertical</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/crucial-conversations-book-rec-2026-03-27/crucial-conversations-7-skills</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G157" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>STATE method: Share facts, Tell story, Ask others paths, Talk tentatively, Encourage testing</t>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Book rec carousel. No people tagged.</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>crucial-conversations-crib-technique</t>
+          <t>crucial-conversations-apply</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Crucial Conversations by Patterson et al</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>square, portrait, vertical</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/crucial-conversations-book-rec-2026-03-27/crucial-conversations-apply</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>CRIB technique: Commit, Recognize, Invent, Brainstorm for finding mutual purpose</t>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>Book rec carousel. No people tagged.</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>best-teacher-resigned-warning-signs</t>
+          <t>teacher-resigned-what-happened</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Your Best Teacher Just Resigned</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>square, portrait, vertical</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/best-teacher-resigned-2026-03-27/teacher-resigned-what-happened</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>5 warning signs you missed, 75% stat, stay conversation advice</t>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>Pain point carousel about teacher retention.</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>best-teacher-resigned-why-they-leave</t>
+          <t>teacher-resigned-warning-signs</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Your Best Teacher Just Resigned</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>square, portrait, vertical</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/best-teacher-resigned-2026-03-27/teacher-resigned-warning-signs</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G160" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>Real reasons: invisible, bureaucracy, no voice, toxic culture, no future. $10-20K cost per teacher</t>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>Pain point carousel about teacher retention.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>best-teacher-resigned-how-to-keep</t>
+          <t>teacher-resigned-how-to-keep</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Your Best Teacher Just Resigned</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="D161" t="n">
+        <v>8</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/best-teacher-resigned-2026-03-27/teacher-resigned-how-to-keep</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Pain point carousel about teacher retention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>dare-to-lead-why-listen</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>8</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/dare-to-lead-podcast-rec-2026-03-27/dare-to-lead-why-listen</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>Podcast rec carousel for Dare to Lead with Brene Brown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>dare-to-lead-key-themes</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
         <v>7</v>
       </c>
-      <c r="E161" t="inlineStr">
-        <is>
-          <t>square, portrait, vertical</t>
-        </is>
-      </c>
-      <c r="F161" t="inlineStr">
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/dare-to-lead-podcast-rec-2026-03-27/dare-to-lead-key-themes</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>Podcast rec carousel for Dare to Lead with Brene Brown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>board-offsite-why</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="G161" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
-        </is>
-      </c>
-      <c r="H161" t="inlineStr">
-        <is>
-          <t>6 strategies: relationships, voice, growth, protect time. 2/3 nobody asked them to stay</t>
+      <c r="D164" t="n">
+        <v>8</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/board-offsite-nonprofits-2026-03-27/board-offsite-why</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>Service carousel for Board Offsite for Nonprofits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>board-offsite-5-signs</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>7</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/board-offsite-nonprofits-2026-03-27/board-offsite-5-signs</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>Service carousel for Board Offsite for Nonprofits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>The Pre-Brief Call</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>8</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/pre-brief-zoom-call-2026-03-27/pre-brief-call</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>Behind the scenes carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>5 Questions Before Every Offsite</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>8</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/pre-brief-zoom-call-2026-03-27/5-questions-before-offsite</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>Behind the scenes carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>What Is Vulnerability-Based Trust?</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/vulnerability-based-trust</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>8</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/vulnerability-based-trust-2026-03-27/what-is-vulnerability-based-trust</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>Concept overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>7 Ways to Build Vulnerability-Based Trust</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/vulnerability-based-trust</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>9</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/vulnerability-based-trust-2026-03-27/7-ways-vulnerability-trust</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>Practical tips</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>The Leader Must Go First</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/vulnerability-based-trust</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>8</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/vulnerability-based-trust-2026-03-27/leader-must-go-first</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>Leadership role in trust</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Why Every Leader Should Read Atomic Habits</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>8</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/atomic-habits-2026-03-27/atomic-habits-book-rec</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>Book rec carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>The 4 Laws of Behaviour Change</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>8</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/atomic-habits-2026-03-27/4-laws-behaviour-change</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>Book rec carousel - framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>We Did an Offsite and Nothing Changed</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>8</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/offsite-nothing-changed-2026-03-27/offsite-nothing-changed</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>Pain point carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>3 Signs Your Offsite Will Fail</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>7</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/offsite-nothing-changed-2026-03-27/3-signs-offsite-fail</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>Pain point carousel - warning signs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update carousel log — 8 carousels added 2026-03-27
</commit_message>
<xml_diff>
--- a/carousel-data/carousel-log.xlsx
+++ b/carousel-data/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K199"/>
+  <dimension ref="A1:K200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10523,7 +10523,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>school-pd-day-what-2026-03-27</t>
+          <t>school-pd-day-reasons</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -10531,27 +10531,23 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C193" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/school-leadership-pd-day</t>
-        </is>
-      </c>
+      <c r="C193" t="inlineStr"/>
       <c r="D193" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/school-pd-day-what-2026-03-27</t>
+          <t>carousels/school-leadership-pd-day-2026-03-27/school-pd-day-reasons</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>YouTube (queue full)</t>
+          <t>IG tags, X tags</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
@@ -10566,19 +10562,19 @@
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>Yes (Pinterest skipped)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>Topic 1A of 4</t>
+          <t>Service: School Leadership PD Day</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>school-pd-day-why-2026-03-27</t>
+          <t>school-pd-day-agenda</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -10586,27 +10582,23 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C194" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/school-leadership-pd-day</t>
-        </is>
-      </c>
+      <c r="C194" t="inlineStr"/>
       <c r="D194" t="n">
         <v>8</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/school-pd-day-why-2026-03-27</t>
+          <t>carousels/school-leadership-pd-day-2026-03-27/school-pd-day-agenda</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>YouTube (queue full)</t>
+          <t>IG tags, X tags</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
@@ -10621,19 +10613,19 @@
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>Yes (Pinterest skipped)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
         <is>
-          <t>Topic 1B of 4</t>
+          <t>Service: School Leadership PD Day</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>step-up-framework-2026-03-27</t>
+          <t>step-up-framework</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -10641,27 +10633,23 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/step-up-or-step-out-the-framework</t>
-        </is>
-      </c>
+      <c r="C195" t="inlineStr"/>
       <c r="D195" t="n">
         <v>8</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/step-up-framework-2026-03-27</t>
+          <t>carousels/step-up-or-step-out-framework-2026-03-27/step-up-framework</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>Instagram, Google Business, TikTok, Bluesky</t>
+          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>YouTube (queue full); LinkedIn, Facebook, Threads, X/Twitter (duplicate detected)</t>
+          <t>IG tags, X tags</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
@@ -10676,19 +10664,19 @@
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>Yes (Pinterest skipped)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>Topic 2A - some platforms rejected as duplicate</t>
+          <t>Framework: Step Up or Step Out</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>step-up-signs-2026-03-27</t>
+          <t>step-up-signs</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -10696,27 +10684,23 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C196" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/step-up-or-step-out-the-framework</t>
-        </is>
-      </c>
+      <c r="C196" t="inlineStr"/>
       <c r="D196" t="n">
         <v>7</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/step-up-signs-2026-03-27</t>
+          <t>carousels/step-up-or-step-out-framework-2026-03-27/step-up-signs</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>YouTube (queue full)</t>
+          <t>IG tags, X tags</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
@@ -10731,19 +10715,19 @@
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>Yes (Pinterest skipped)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
         <is>
-          <t>Topic 2B of 4</t>
+          <t>Framework: Step Up or Step Out</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>personal-histories-2026-03-27</t>
+          <t>personal-histories-what</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -10751,27 +10735,23 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/the-personal-histories-exercise</t>
-        </is>
-      </c>
+      <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
         <v>8</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/personal-histories-2026-03-27</t>
+          <t>carousels/personal-histories-exercise-2026-03-27/personal-histories-what</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>YouTube (queue full)</t>
+          <t>IG tags, X tags</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
@@ -10786,19 +10766,19 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>Yes (Pinterest skipped)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>Topic 3A of 4</t>
+          <t>Blog: The Personal Histories Exercise</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>personal-histories-how-2026-03-27</t>
+          <t>personal-histories-why</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -10806,27 +10786,23 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/the-personal-histories-exercise</t>
-        </is>
-      </c>
+      <c r="C198" t="inlineStr"/>
       <c r="D198" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/personal-histories-how-2026-03-27</t>
+          <t>carousels/personal-histories-exercise-2026-03-27/personal-histories-why</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>YouTube (queue full)</t>
+          <t>IG tags, X tags</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
@@ -10841,19 +10817,19 @@
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>Yes (Pinterest skipped)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
         <is>
-          <t>Topic 3B of 4</t>
+          <t>Blog: The Personal Histories Exercise</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>ideal-team-player-2026-03-27</t>
+          <t>ideal-team-player-book</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -10861,32 +10837,28 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C199" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/the-ideal-team-player</t>
-        </is>
-      </c>
+      <c r="C199" t="inlineStr"/>
       <c r="D199" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/ideal-team-player-2026-03-27</t>
+          <t>carousels/ideal-team-player-book-rec-2026-03-27/ideal-team-player-book</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>YouTube (queue full)</t>
+          <t>IG tags, X tags</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>Author | Keynote Speaker</t>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -10896,12 +10868,63 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>Yes (Pinterest skipped)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>Topic 4 of 4</t>
+          <t>Book Rec: The Ideal Team Player</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>ideal-team-player-missing</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr"/>
+      <c r="D200" t="n">
+        <v>8</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>carousels/ideal-team-player-book-rec-2026-03-27/ideal-team-player-missing</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>IG tags, X tags</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>Book Rec: The Ideal Team Player</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update carousel log - 8 new carousels (rows 193-200)
</commit_message>
<xml_diff>
--- a/carousel-data/carousel-log.xlsx
+++ b/carousel-data/carousel-log.xlsx
@@ -10523,7 +10523,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>school-pd-day-reasons</t>
+          <t>what-a-pd-day-looks-like</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -10531,23 +10531,27 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C193" t="inlineStr"/>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>N/A - service page</t>
+        </is>
+      </c>
       <c r="D193" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>carousels/school-leadership-pd-day-2026-03-27/school-pd-day-reasons</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/school-leadership-pd-day-2026-03-27/what-a-pd-day-looks-like</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>IG tags, X tags</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
@@ -10562,19 +10566,15 @@
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K193" t="inlineStr">
-        <is>
-          <t>Service: School Leadership PD Day</t>
-        </is>
-      </c>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>school-pd-day-agenda</t>
+          <t>why-book-jonno-pd-day</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -10582,23 +10582,27 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C194" t="inlineStr"/>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>N/A - service page</t>
+        </is>
+      </c>
       <c r="D194" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>carousels/school-leadership-pd-day-2026-03-27/school-pd-day-agenda</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/school-leadership-pd-day-2026-03-27/why-book-jonno-pd-day</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>IG tags, X tags</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
@@ -10613,19 +10617,15 @@
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K194" t="inlineStr">
-        <is>
-          <t>Service: School Leadership PD Day</t>
-        </is>
-      </c>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>step-up-framework</t>
+          <t>step-up-step-out-framework</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -10633,28 +10633,32 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr"/>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>N/A - framework</t>
+        </is>
+      </c>
       <c r="D195" t="n">
         <v>8</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>carousels/step-up-or-step-out-framework-2026-03-27/step-up-framework</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/step-up-step-out-2026-03-27/step-up-step-out-framework</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>IG tags, X tags</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>Author | Keynote Speaker</t>
+          <t>Leadership Team Facilitator | Author</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -10664,19 +10668,15 @@
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K195" t="inlineStr">
-        <is>
-          <t>Framework: Step Up or Step Out</t>
-        </is>
-      </c>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>step-up-signs</t>
+          <t>5-signs-have-conversation</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -10684,28 +10684,32 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C196" t="inlineStr"/>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>N/A - framework</t>
+        </is>
+      </c>
       <c r="D196" t="n">
         <v>7</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>carousels/step-up-or-step-out-framework-2026-03-27/step-up-signs</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/step-up-step-out-2026-03-27/5-signs-have-conversation</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>IG tags, X tags</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>Author | Keynote Speaker</t>
+          <t>Leadership Team Facilitator | Author</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -10715,19 +10719,15 @@
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K196" t="inlineStr">
-        <is>
-          <t>Framework: Step Up or Step Out</t>
-        </is>
-      </c>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>personal-histories-what</t>
+          <t>build-trust-30-minutes</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -10735,28 +10735,32 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr"/>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>N/A - blog</t>
+        </is>
+      </c>
       <c r="D197" t="n">
         <v>8</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>carousels/personal-histories-exercise-2026-03-27/personal-histories-what</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/personal-histories-exercise-2026-03-27/build-trust-30-minutes</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>IG tags, X tags</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+          <t>Leadership Team Facilitator | Author</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -10766,19 +10770,15 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K197" t="inlineStr">
-        <is>
-          <t>Blog: The Personal Histories Exercise</t>
-        </is>
-      </c>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>personal-histories-why</t>
+          <t>how-to-run-personal-histories</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -10786,28 +10786,32 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C198" t="inlineStr"/>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>N/A - blog</t>
+        </is>
+      </c>
       <c r="D198" t="n">
         <v>7</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>carousels/personal-histories-exercise-2026-03-27/personal-histories-why</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/personal-histories-exercise-2026-03-27/how-to-run-personal-histories</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>IG tags, X tags</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+          <t>Leadership Team Facilitator | Author</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -10817,14 +10821,10 @@
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K198" t="inlineStr">
-        <is>
-          <t>Blog: The Personal Histories Exercise</t>
-        </is>
-      </c>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -10837,28 +10837,32 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C199" t="inlineStr"/>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>N/A - book rec</t>
+        </is>
+      </c>
       <c r="D199" t="n">
         <v>8</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>carousels/ideal-team-player-book-rec-2026-03-27/ideal-team-player-book</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/ideal-team-player-book-rec-2026-03-27/ideal-team-player-book</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>IG tags, X tags</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+          <t>Leadership Team Facilitator | Author</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -10868,19 +10872,15 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K199" t="inlineStr">
-        <is>
-          <t>Book Rec: The Ideal Team Player</t>
-        </is>
-      </c>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>ideal-team-player-missing</t>
+          <t>are-you-ideal-team-player</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -10888,28 +10888,32 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C200" t="inlineStr"/>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>N/A - book rec</t>
+        </is>
+      </c>
       <c r="D200" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>carousels/ideal-team-player-book-rec-2026-03-27/ideal-team-player-missing</t>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/ideal-team-player-book-rec-2026-03-27/are-you-ideal-team-player</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>LI,FB,IG,Threads,X,GBP,Bluesky,TikTok,YouTube</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>IG tags, X tags</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+          <t>Leadership Team Facilitator | Author</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -10919,14 +10923,10 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K200" t="inlineStr">
-        <is>
-          <t>Book Rec: The Ideal Team Player</t>
-        </is>
-      </c>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>

</xml_diff>